<commit_message>
update the variable list file
</commit_message>
<xml_diff>
--- a/fps_convection_variables_vfinal_2021update_with_addons.xlsx
+++ b/fps_convection_variables_vfinal_2021update_with_addons.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kgo/Documents/tools/postpro/WRF_CMORizer_my_dev_with_git/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224093AC-A289-C840-9E7C-04FCC67507AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2A7FA7E-8A6D-3041-A786-D4B23B3F5723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1340" yWindow="760" windowWidth="48020" windowHeight="28040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Core" sheetId="4" r:id="rId1"/>
@@ -5171,23 +5171,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="15" fontId="15" fillId="2" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="15" fillId="2" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="135">
@@ -5723,17 +5723,17 @@
   <dimension ref="A1:AF158"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="6" width="25" style="56" customWidth="1"/>
-    <col min="7" max="7" width="25" style="7" customWidth="1"/>
-    <col min="8" max="9" width="25" style="56" customWidth="1"/>
+    <col min="1" max="6" width="25" style="56" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="25" style="7" hidden="1" customWidth="1"/>
+    <col min="8" max="9" width="25" style="56" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="12" width="10.83203125" customWidth="1"/>
-    <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="11.83203125" customWidth="1"/>
-    <col min="15" max="15" width="10.83203125" customWidth="1"/>
-    <col min="16" max="16" width="23.6640625" customWidth="1"/>
+    <col min="11" max="12" width="10.83203125" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="13" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="11.83203125" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="10.83203125" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="23.6640625" hidden="1" customWidth="1"/>
     <col min="17" max="17" width="32.1640625" customWidth="1"/>
-    <col min="18" max="22" width="23.6640625" customWidth="1"/>
+    <col min="18" max="22" width="23.6640625" hidden="1" customWidth="1"/>
     <col min="26" max="27" width="10" style="10" customWidth="1"/>
     <col min="28" max="28" width="18.83203125" customWidth="1"/>
   </cols>
@@ -11234,12 +11234,14 @@
   <dimension ref="A1:AD22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="7" width="27.5" style="56" customWidth="1"/>
+    <col min="1" max="7" width="27.5" style="56" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" customWidth="1"/>
-    <col min="14" max="14" width="23.6640625" customWidth="1"/>
+    <col min="9" max="11" width="0" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="0" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="23.6640625" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="33" customWidth="1"/>
-    <col min="16" max="20" width="23.6640625" customWidth="1"/>
+    <col min="16" max="20" width="23.6640625" hidden="1" customWidth="1"/>
     <col min="24" max="25" width="10" style="10" customWidth="1"/>
     <col min="26" max="26" width="18.83203125" customWidth="1"/>
   </cols>
@@ -12678,22 +12680,22 @@
       <c r="D2" s="92" t="s">
         <v>259</v>
       </c>
-      <c r="E2" s="306" t="str">
+      <c r="E2" s="304" t="str">
         <f>[1]all!R5</f>
         <v>10 Feb 2014 Version 3.1</v>
       </c>
-      <c r="F2" s="306"/>
-      <c r="G2" s="306"/>
-      <c r="H2" s="306"/>
-      <c r="I2" s="306"/>
-      <c r="J2" s="306"/>
-      <c r="K2" s="306"/>
-      <c r="L2" s="306"/>
-      <c r="M2" s="306"/>
-      <c r="N2" s="306"/>
-      <c r="O2" s="306"/>
-      <c r="P2" s="306"/>
-      <c r="Q2" s="306"/>
+      <c r="F2" s="304"/>
+      <c r="G2" s="304"/>
+      <c r="H2" s="304"/>
+      <c r="I2" s="304"/>
+      <c r="J2" s="304"/>
+      <c r="K2" s="304"/>
+      <c r="L2" s="304"/>
+      <c r="M2" s="304"/>
+      <c r="N2" s="304"/>
+      <c r="O2" s="304"/>
+      <c r="P2" s="304"/>
+      <c r="Q2" s="304"/>
     </row>
     <row r="3" spans="1:17" s="100" customFormat="1">
       <c r="A3" s="93" t="s">
@@ -12706,10 +12708,10 @@
       <c r="D3" s="95" t="s">
         <v>261</v>
       </c>
-      <c r="E3" s="307" t="s">
+      <c r="E3" s="305" t="s">
         <v>262</v>
       </c>
-      <c r="F3" s="307"/>
+      <c r="F3" s="305"/>
       <c r="G3" s="96"/>
       <c r="H3" s="96"/>
       <c r="I3" s="96"/>
@@ -12760,13 +12762,13 @@
       <c r="D5" s="108" t="s">
         <v>261</v>
       </c>
-      <c r="E5" s="308" t="s">
+      <c r="E5" s="306" t="s">
         <v>263</v>
       </c>
-      <c r="F5" s="308"/>
-      <c r="G5" s="308"/>
-      <c r="H5" s="308"/>
-      <c r="I5" s="308"/>
+      <c r="F5" s="306"/>
+      <c r="G5" s="306"/>
+      <c r="H5" s="306"/>
+      <c r="I5" s="306"/>
       <c r="J5" s="109"/>
       <c r="K5" s="109"/>
       <c r="L5" s="109"/>
@@ -12810,12 +12812,12 @@
       <c r="K6" s="102" t="s">
         <v>273</v>
       </c>
-      <c r="L6" s="309"/>
-      <c r="M6" s="309"/>
-      <c r="N6" s="309"/>
-      <c r="O6" s="309"/>
-      <c r="P6" s="309"/>
-      <c r="Q6" s="309"/>
+      <c r="L6" s="307"/>
+      <c r="M6" s="307"/>
+      <c r="N6" s="307"/>
+      <c r="O6" s="307"/>
+      <c r="P6" s="307"/>
+      <c r="Q6" s="307"/>
     </row>
     <row r="7" spans="1:17" s="100" customFormat="1" ht="17">
       <c r="A7" s="101" t="s">
@@ -12979,16 +12981,16 @@
       <c r="F12" s="102" t="s">
         <v>290</v>
       </c>
-      <c r="G12" s="304" t="s">
+      <c r="G12" s="308" t="s">
         <v>291</v>
       </c>
-      <c r="H12" s="304"/>
-      <c r="I12" s="304"/>
-      <c r="J12" s="304"/>
-      <c r="K12" s="304"/>
-      <c r="L12" s="304"/>
-      <c r="M12" s="304"/>
-      <c r="N12" s="304"/>
+      <c r="H12" s="308"/>
+      <c r="I12" s="308"/>
+      <c r="J12" s="308"/>
+      <c r="K12" s="308"/>
+      <c r="L12" s="308"/>
+      <c r="M12" s="308"/>
+      <c r="N12" s="308"/>
       <c r="O12" s="105"/>
       <c r="P12" s="105"/>
       <c r="Q12" s="106"/>
@@ -13167,12 +13169,12 @@
       <c r="D18" s="118" t="s">
         <v>284</v>
       </c>
-      <c r="E18" s="305" t="s">
+      <c r="E18" s="309" t="s">
         <v>316</v>
       </c>
-      <c r="F18" s="305"/>
-      <c r="G18" s="305"/>
-      <c r="H18" s="305"/>
+      <c r="F18" s="309"/>
+      <c r="G18" s="309"/>
+      <c r="H18" s="309"/>
       <c r="I18" s="117"/>
       <c r="J18" s="117"/>
       <c r="K18" s="117"/>
@@ -13190,17 +13192,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="E11:I11"/>
+    <mergeCell ref="G12:N12"/>
+    <mergeCell ref="E13:J13"/>
+    <mergeCell ref="E17:M17"/>
+    <mergeCell ref="E18:H18"/>
     <mergeCell ref="E10:N10"/>
     <mergeCell ref="E2:Q2"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="E4:I4"/>
     <mergeCell ref="E5:I5"/>
     <mergeCell ref="L6:Q6"/>
-    <mergeCell ref="E11:I11"/>
-    <mergeCell ref="G12:N12"/>
-    <mergeCell ref="E13:J13"/>
-    <mergeCell ref="E17:M17"/>
-    <mergeCell ref="E18:H18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>